<commit_message>
Modificar urls y views
</commit_message>
<xml_diff>
--- a/docs/base-datos/matriz datos documentos.xlsx
+++ b/docs/base-datos/matriz datos documentos.xlsx
@@ -5,16 +5,19 @@
   <workbookPr defaultThemeVersion="164011"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\SOFIA\ESTUDIOS\UNIVERSIDADES\UIS\PROYECTOS GITHUB\sistema-auditoria\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\SOFIA\ESTUDIOS\UNIVERSIDADES\UIS\PROYECTOS GITHUB\sistema-auditoria\docs\base-datos\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="15288" windowHeight="4524"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="15288" windowHeight="4524" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="Matriz" sheetId="2" r:id="rId1"/>
     <sheet name="Borrador" sheetId="1" r:id="rId2"/>
   </sheets>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">Borrador!$A$4:$E$46</definedName>
+  </definedNames>
   <calcPr calcId="162913"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
@@ -917,6 +920,9 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
@@ -925,9 +931,6 @@
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1263,25 +1266,25 @@
   </cols>
   <sheetData>
     <row r="2" spans="1:7" ht="42" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="12" t="s">
+      <c r="A2" s="9" t="s">
         <v>47</v>
       </c>
-      <c r="B2" s="12" t="s">
+      <c r="B2" s="9" t="s">
         <v>2</v>
       </c>
-      <c r="C2" s="12" t="s">
+      <c r="C2" s="9" t="s">
         <v>3</v>
       </c>
-      <c r="D2" s="12" t="s">
+      <c r="D2" s="9" t="s">
         <v>48</v>
       </c>
-      <c r="E2" s="12" t="s">
+      <c r="E2" s="9" t="s">
         <v>4</v>
       </c>
-      <c r="F2" s="12" t="s">
+      <c r="F2" s="9" t="s">
         <v>49</v>
       </c>
-      <c r="G2" s="12" t="s">
+      <c r="G2" s="9" t="s">
         <v>50</v>
       </c>
     </row>
@@ -1608,26 +1611,26 @@
       </c>
     </row>
     <row r="17" spans="1:7" ht="43.2" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A17" s="10" t="s">
+      <c r="A17" s="11" t="s">
         <v>89</v>
       </c>
-      <c r="B17" s="10"/>
-      <c r="C17" s="10"/>
-      <c r="D17" s="10"/>
-      <c r="E17" s="10"/>
-      <c r="F17" s="10"/>
-      <c r="G17" s="10"/>
+      <c r="B17" s="11"/>
+      <c r="C17" s="11"/>
+      <c r="D17" s="11"/>
+      <c r="E17" s="11"/>
+      <c r="F17" s="11"/>
+      <c r="G17" s="11"/>
     </row>
     <row r="18" spans="1:7" ht="30.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A18" s="9" t="s">
+      <c r="A18" s="10" t="s">
         <v>90</v>
       </c>
-      <c r="B18" s="9"/>
-      <c r="C18" s="9"/>
-      <c r="D18" s="9"/>
-      <c r="E18" s="9"/>
-      <c r="F18" s="9"/>
-      <c r="G18" s="9"/>
+      <c r="B18" s="10"/>
+      <c r="C18" s="10"/>
+      <c r="D18" s="10"/>
+      <c r="E18" s="10"/>
+      <c r="F18" s="10"/>
+      <c r="G18" s="10"/>
     </row>
     <row r="19" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A19" s="3" t="s">
@@ -1791,15 +1794,15 @@
       </c>
     </row>
     <row r="26" spans="1:7" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A26" s="9" t="s">
+      <c r="A26" s="10" t="s">
         <v>110</v>
       </c>
-      <c r="B26" s="9"/>
-      <c r="C26" s="9"/>
-      <c r="D26" s="9"/>
-      <c r="E26" s="9"/>
-      <c r="F26" s="9"/>
-      <c r="G26" s="9"/>
+      <c r="B26" s="10"/>
+      <c r="C26" s="10"/>
+      <c r="D26" s="10"/>
+      <c r="E26" s="10"/>
+      <c r="F26" s="10"/>
+      <c r="G26" s="10"/>
     </row>
     <row r="27" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A27" s="3" t="s">
@@ -2032,15 +2035,15 @@
       </c>
     </row>
     <row r="37" spans="1:7" ht="25.8" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A37" s="9" t="s">
+      <c r="A37" s="10" t="s">
         <v>129</v>
       </c>
-      <c r="B37" s="9"/>
-      <c r="C37" s="9"/>
-      <c r="D37" s="9"/>
-      <c r="E37" s="9"/>
-      <c r="F37" s="9"/>
-      <c r="G37" s="9"/>
+      <c r="B37" s="10"/>
+      <c r="C37" s="10"/>
+      <c r="D37" s="10"/>
+      <c r="E37" s="10"/>
+      <c r="F37" s="10"/>
+      <c r="G37" s="10"/>
     </row>
     <row r="38" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A38" s="3" t="s">
@@ -2158,15 +2161,15 @@
       </c>
     </row>
     <row r="43" spans="1:7" ht="29.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A43" s="9" t="s">
+      <c r="A43" s="10" t="s">
         <v>138</v>
       </c>
-      <c r="B43" s="9"/>
-      <c r="C43" s="9"/>
-      <c r="D43" s="9"/>
-      <c r="E43" s="9"/>
-      <c r="F43" s="9"/>
-      <c r="G43" s="9"/>
+      <c r="B43" s="10"/>
+      <c r="C43" s="10"/>
+      <c r="D43" s="10"/>
+      <c r="E43" s="10"/>
+      <c r="F43" s="10"/>
+      <c r="G43" s="10"/>
     </row>
     <row r="44" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A44" s="3" t="s">
@@ -2537,15 +2540,15 @@
       </c>
     </row>
     <row r="60" spans="1:7" ht="28.8" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A60" s="9" t="s">
+      <c r="A60" s="10" t="s">
         <v>162</v>
       </c>
-      <c r="B60" s="9"/>
-      <c r="C60" s="9"/>
-      <c r="D60" s="9"/>
-      <c r="E60" s="9"/>
-      <c r="F60" s="9"/>
-      <c r="G60" s="9"/>
+      <c r="B60" s="10"/>
+      <c r="C60" s="10"/>
+      <c r="D60" s="10"/>
+      <c r="E60" s="10"/>
+      <c r="F60" s="10"/>
+      <c r="G60" s="10"/>
     </row>
     <row r="61" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A61" s="3" t="s">
@@ -2732,15 +2735,15 @@
       </c>
     </row>
     <row r="69" spans="1:7" ht="32.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A69" s="9" t="s">
+      <c r="A69" s="10" t="s">
         <v>178</v>
       </c>
-      <c r="B69" s="9"/>
-      <c r="C69" s="9"/>
-      <c r="D69" s="9"/>
-      <c r="E69" s="9"/>
-      <c r="F69" s="9"/>
-      <c r="G69" s="9"/>
+      <c r="B69" s="10"/>
+      <c r="C69" s="10"/>
+      <c r="D69" s="10"/>
+      <c r="E69" s="10"/>
+      <c r="F69" s="10"/>
+      <c r="G69" s="10"/>
     </row>
     <row r="70" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A70" s="3" t="s">
@@ -2858,15 +2861,15 @@
       </c>
     </row>
     <row r="75" spans="1:7" ht="35.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A75" s="9" t="s">
+      <c r="A75" s="10" t="s">
         <v>184</v>
       </c>
-      <c r="B75" s="9"/>
-      <c r="C75" s="9"/>
-      <c r="D75" s="9"/>
-      <c r="E75" s="9"/>
-      <c r="F75" s="9"/>
-      <c r="G75" s="9"/>
+      <c r="B75" s="10"/>
+      <c r="C75" s="10"/>
+      <c r="D75" s="10"/>
+      <c r="E75" s="10"/>
+      <c r="F75" s="10"/>
+      <c r="G75" s="10"/>
     </row>
     <row r="76" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A76" s="3" t="s">
@@ -3099,15 +3102,15 @@
       </c>
     </row>
     <row r="86" spans="1:7" ht="43.2" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A86" s="9" t="s">
+      <c r="A86" s="10" t="s">
         <v>201</v>
       </c>
-      <c r="B86" s="9"/>
-      <c r="C86" s="9"/>
-      <c r="D86" s="9"/>
-      <c r="E86" s="9"/>
-      <c r="F86" s="9"/>
-      <c r="G86" s="9"/>
+      <c r="B86" s="10"/>
+      <c r="C86" s="10"/>
+      <c r="D86" s="10"/>
+      <c r="E86" s="10"/>
+      <c r="F86" s="10"/>
+      <c r="G86" s="10"/>
     </row>
     <row r="87" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A87" s="3" t="s">
@@ -3294,15 +3297,15 @@
       </c>
     </row>
     <row r="95" spans="1:7" ht="32.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A95" s="9" t="s">
+      <c r="A95" s="10" t="s">
         <v>213</v>
       </c>
-      <c r="B95" s="9"/>
-      <c r="C95" s="9"/>
-      <c r="D95" s="9"/>
-      <c r="E95" s="9"/>
-      <c r="F95" s="9"/>
-      <c r="G95" s="9"/>
+      <c r="B95" s="10"/>
+      <c r="C95" s="10"/>
+      <c r="D95" s="10"/>
+      <c r="E95" s="10"/>
+      <c r="F95" s="10"/>
+      <c r="G95" s="10"/>
     </row>
     <row r="96" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A96" s="3" t="s">
@@ -3419,15 +3422,15 @@
       <c r="G101" s="7"/>
     </row>
     <row r="102" spans="1:7" ht="37.200000000000003" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A102" s="9" t="s">
+      <c r="A102" s="10" t="s">
         <v>224</v>
       </c>
-      <c r="B102" s="9"/>
-      <c r="C102" s="9"/>
-      <c r="D102" s="9"/>
-      <c r="E102" s="9"/>
-      <c r="F102" s="9"/>
-      <c r="G102" s="9"/>
+      <c r="B102" s="10"/>
+      <c r="C102" s="10"/>
+      <c r="D102" s="10"/>
+      <c r="E102" s="10"/>
+      <c r="F102" s="10"/>
+      <c r="G102" s="10"/>
     </row>
     <row r="103" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A103" s="3" t="s">
@@ -3559,17 +3562,17 @@
     </row>
   </sheetData>
   <mergeCells count="11">
+    <mergeCell ref="A69:G69"/>
+    <mergeCell ref="A75:G75"/>
+    <mergeCell ref="A86:G86"/>
+    <mergeCell ref="A95:G95"/>
+    <mergeCell ref="A102:G102"/>
     <mergeCell ref="A60:G60"/>
     <mergeCell ref="A17:G17"/>
     <mergeCell ref="A18:G18"/>
     <mergeCell ref="A26:G26"/>
     <mergeCell ref="A37:G37"/>
     <mergeCell ref="A43:G43"/>
-    <mergeCell ref="A69:G69"/>
-    <mergeCell ref="A75:G75"/>
-    <mergeCell ref="A86:G86"/>
-    <mergeCell ref="A95:G95"/>
-    <mergeCell ref="A102:G102"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
@@ -3590,13 +3593,13 @@
   </cols>
   <sheetData>
     <row r="3" spans="1:9" ht="22.2" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="11" t="s">
+      <c r="A3" s="12" t="s">
         <v>0</v>
       </c>
-      <c r="B3" s="11"/>
-      <c r="C3" s="11"/>
-      <c r="D3" s="11"/>
-      <c r="E3" s="11"/>
+      <c r="B3" s="12"/>
+      <c r="C3" s="12"/>
+      <c r="D3" s="12"/>
+      <c r="E3" s="12"/>
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A4" s="5" t="s">
@@ -4146,6 +4149,7 @@
       </c>
     </row>
   </sheetData>
+  <autoFilter ref="A4:E46"/>
   <mergeCells count="1">
     <mergeCell ref="A3:E3"/>
   </mergeCells>

</xml_diff>